<commit_message>
se agrega convell hull sobre los clientes
</commit_message>
<xml_diff>
--- a/public/templates/Formato_excel_clientes.xlsx
+++ b/public/templates/Formato_excel_clientes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desarrollo\React\Convex Hull\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66698198-D97E-4727-9348-0A07941BF4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4BBF490-E096-444E-BABC-88CA333FA91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
@@ -1067,7 +1067,7 @@
         <v>37</v>
       </c>
       <c r="C15">
-        <v>20.491541000000002</v>
+        <v>19.491541000000002</v>
       </c>
       <c r="D15">
         <v>-99.731881000000001</v>

</xml_diff>